<commit_message>
default headers to bold
</commit_message>
<xml_diff>
--- a/src/ExcelsiorClosedXml.Tests/ColumnAttributeTests.Test.verified.xlsx
+++ b/src/ExcelsiorClosedXml.Tests/ColumnAttributeTests.Test.verified.xlsx
@@ -54,8 +54,16 @@
     <x:numFmt numFmtId="164" formatCode="0000"/>
     <x:numFmt numFmtId="165" formatCode="yyyy-MM-dd"/>
   </x:numFmts>
-  <x:fonts count="1">
+  <x:fonts count="2">
     <x:font>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
+      <x:b/>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
       <x:color rgb="FF000000"/>
@@ -90,10 +98,13 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="3">
+  <x:cellStyleXfs count="4">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -101,8 +112,12 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -423,44 +438,44 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:4" ht="14.25" customHeight="1">
-      <x:c r="A1" s="0" t="s">
+      <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
+      <x:c r="B1" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C1" s="0" t="s">
+      <x:c r="C1" s="1" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D1" s="0" t="s">
+      <x:c r="D1" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4" ht="14.25" customHeight="1">
-      <x:c r="A2" s="1">
+      <x:c r="A2" s="2">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="s">
+      <x:c r="B2" s="3" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C2" s="3">
+      <x:c r="C2" s="4">
         <x:v>43845</x:v>
       </x:c>
-      <x:c r="D2" s="2" t="s">
+      <x:c r="D2" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4" ht="14.25" customHeight="1">
-      <x:c r="A3" s="1">
+      <x:c r="A3" s="2">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
+      <x:c r="B3" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C3" s="2" t="s">
+      <x:c r="C3" s="3" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D3" s="2" t="s">
+      <x:c r="D3" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
     </x:row>

</xml_diff>